<commit_message>
Implement reviewed card redesign and preserve pending effects
</commit_message>
<xml_diff>
--- a/design/editable/card-editing.xlsx
+++ b/design/editable/card-editing.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>PEAK target: 2.6.b. Source: design/cards.json, mod 0.5.1. All 64 cards are included.</t>
+          <t>PEAK target: 2.6.b. Source: design/cards.json, mod 0.6.0. All 64 cards are included. See card-edit-review.xlsx for your submitted requests and their implementation status.</t>
         </is>
       </c>
     </row>
@@ -539,7 +539,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Notes flag known limitations. Current code shows the actual modifiers, ability handler and parameters. PackRat is disabled by default.</t>
+          <t>Notes flag known limitations. Current code shows the actual modifiers, ability handler and parameters. Existing Enabled settings are preserved during upgrade.</t>
         </is>
       </c>
     </row>
@@ -689,15 +689,19 @@
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>Piton-Free Fingers</t>
+          <t>Piton Fingers</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>Climbing tires you 12% less.</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr"/>
+          <t>Lose stamina 12% slower when climbing.</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Sprinting stamina drains 12% faster</t>
+        </is>
+      </c>
       <c r="I2" s="6" t="inlineStr"/>
       <c r="J2" s="6" t="inlineStr"/>
       <c r="K2" s="4" t="inlineStr"/>
@@ -728,7 +732,7 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>Budget Scout Cannon</t>
+          <t>Mini Scout Cannon</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
@@ -771,15 +775,19 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Swipity, No Slippity</t>
+          <t>To The Bone</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>You slip and slide 35% less.</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr"/>
+          <t>You take 35% less cold when climbing on blue ice.</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Takes 10% longer to warm back up.</t>
+        </is>
+      </c>
       <c r="I4" s="6" t="inlineStr"/>
       <c r="J4" s="6" t="inlineStr"/>
       <c r="K4" s="4" t="inlineStr"/>
@@ -818,7 +826,11 @@
           <t>Hang still on a wall to get 4 stamina back every second.</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Climbing speed is reduced by 30%</t>
+        </is>
+      </c>
       <c r="I5" s="6" t="inlineStr"/>
       <c r="J5" s="6" t="inlineStr"/>
       <c r="K5" s="4" t="inlineStr"/>
@@ -854,7 +866,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Double jump: one extra jump in mid-air, every 35 seconds.</t>
+          <t>Double jump: one extra jump in mid-air. (35 second cooldown)</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -943,7 +955,11 @@
           <t>Falls hurt 25% less.</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr"/>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Dynamite explosions deal 3 times as much Injury.</t>
+        </is>
+      </c>
       <c r="I8" s="6" t="inlineStr"/>
       <c r="J8" s="6" t="inlineStr"/>
       <c r="K8" s="4" t="inlineStr"/>
@@ -974,7 +990,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Myres' Long Arm</t>
+          <t>Daddy</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -982,7 +998,11 @@
           <t>Grab walls from 20% farther away.</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Stamina drains 10% faster.</t>
+        </is>
+      </c>
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
       <c r="K9" s="4" t="inlineStr"/>
@@ -1013,7 +1033,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Scout Cookie Addiction</t>
+          <t>Cookie Addiction</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -1061,13 +1081,17 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Once per biome, when your stamina drops below 20, you get 25 back.</t>
+          <t>Below 20 stamina, press V to restore 25 stamina (5-minute cooldown).</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr"/>
       <c r="I11" s="6" t="inlineStr"/>
       <c r="J11" s="6" t="inlineStr"/>
-      <c r="K11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>Manual V; below 20 stamina, restore 25, five-minute cooldown. Key configurable.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="100" customHeight="1">
       <c r="A12" s="4" t="n">
@@ -1103,7 +1127,11 @@
           <t>Sprinting tires you 15% less.</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Climbing uses 15% more stamina.</t>
+        </is>
+      </c>
       <c r="I12" s="6" t="inlineStr"/>
       <c r="J12" s="6" t="inlineStr"/>
       <c r="K12" s="4" t="inlineStr"/>
@@ -1134,7 +1162,7 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Scout's Microbreak</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -1142,7 +1170,11 @@
           <t>Stamina starts coming back 0.3 seconds sooner.</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr"/>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Stamina bar shrinks 15%</t>
+        </is>
+      </c>
       <c r="I13" s="6" t="inlineStr"/>
       <c r="J13" s="6" t="inlineStr"/>
       <c r="K13" s="4" t="inlineStr"/>
@@ -1173,7 +1205,7 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Gloom Meditation</t>
+          <t>Meditation</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -1181,7 +1213,11 @@
           <t>Crouch and stay still to get stamina back 35% faster.</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Nothing. You're already crouched down staying still</t>
+        </is>
+      </c>
       <c r="I14" s="6" t="inlineStr"/>
       <c r="J14" s="6" t="inlineStr"/>
       <c r="K14" s="4" t="inlineStr"/>
@@ -1212,7 +1248,7 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Myres Made Me Run</t>
+          <t>I'm getting Scoutmastered</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -1255,7 +1291,7 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Endurance Badge Grind</t>
+          <t>Endurance Badge</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -1299,10 +1335,14 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Every time a campfire is lit, get 15 extra (yellow) stamina.</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr"/>
+          <t>Every time a campfire is lit, all your Hunger clears.</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>You can't eat cooked food, even when a teammate feeds you.</t>
+        </is>
+      </c>
       <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="4" t="inlineStr"/>
@@ -1333,17 +1373,17 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Cool Cucumber Complex</t>
+          <t>Cool, Calm, and Collected.</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>You heat up 50% slower.</t>
+          <t>You burn 50% slower.</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>You get cold 30% faster.</t>
+          <t>You freeze 30% faster.</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr"/>
@@ -1376,17 +1416,17 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Bundled Up Badge</t>
+          <t>Just hot.</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>You get cold 50% slower.</t>
+          <t>You freeze 50% slower.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>You heat up 30% faster.</t>
+          <t>You burn 30% faster.</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr"/>
@@ -1427,7 +1467,11 @@
           <t>Poison builds up 35% slower.</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr"/>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>You burn and freeze 25% faster.</t>
+        </is>
+      </c>
       <c r="I20" s="6" t="inlineStr"/>
       <c r="J20" s="6" t="inlineStr"/>
       <c r="K20" s="4" t="inlineStr"/>
@@ -1468,8 +1512,16 @@
       </c>
       <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="inlineStr"/>
-      <c r="J21" s="6" t="inlineStr"/>
-      <c r="K21" s="4" t="inlineStr"/>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>Pending paired replacement: Mandrakes and Zombies do not affect you; a Zombie spawns somewhere random in the next biome.</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>Requested Mandrake/Zombie immunity plus next-biome zombie spawn is pending. The existing spores resistance remains; see docs/card-edit-review.md.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="100" customHeight="1">
       <c r="A22" s="4" t="n">
@@ -1505,7 +1557,11 @@
           <t>New thorns count 40% less.</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr"/>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Takes twice as long to remove the thorns.</t>
+        </is>
+      </c>
       <c r="I22" s="6" t="inlineStr"/>
       <c r="J22" s="6" t="inlineStr"/>
       <c r="K22" s="4" t="inlineStr">
@@ -1540,7 +1596,7 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Aloe Aftercare</t>
+          <t>Aloe</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
@@ -1548,7 +1604,11 @@
           <t>Once you're out of the heat, it wears off 60% faster.</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr"/>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>You burn 15% faster.</t>
+        </is>
+      </c>
       <c r="I23" s="6" t="inlineStr"/>
       <c r="J23" s="6" t="inlineStr"/>
       <c r="K23" s="4" t="inlineStr"/>
@@ -1579,7 +1639,7 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Heat Pack Afterglow</t>
+          <t>Heat Pack</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -1587,7 +1647,11 @@
           <t>Once you're out of the cold, it wears off 60% faster.</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>You freeze 15% faster.</t>
+        </is>
+      </c>
       <c r="I24" s="6" t="inlineStr"/>
       <c r="J24" s="6" t="inlineStr"/>
       <c r="K24" s="4" t="inlineStr"/>
@@ -1623,12 +1687,12 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>While you have 20+ Poison or Spores, climbing tires you 30% less.</t>
+          <t>Above 20 Poison, climbing uses 40% less stamina.</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Poison and Spores wear off 30% slower.</t>
+          <t>Poison wears off 30% slower.</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
@@ -1661,18 +1725,22 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>BingBong Safety Briefing</t>
+          <t>BingBong</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>Hits that aren't falls hurt 20% less.</t>
+          <t>Every 10 minutes while alive, gain Infinite Stamina, Invincibility or Low Gravity for 20 seconds.</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr"/>
       <c r="I26" s="6" t="inlineStr"/>
       <c r="J26" s="6" t="inlineStr"/>
-      <c r="K26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>Native timed Infinite Stamina, Invincibility or Low Gravity. Low Gravity is floating, not free flight. Ghost time pauses the ten-minute clock.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="100" customHeight="1">
       <c r="A27" s="4" t="n">
@@ -1700,7 +1768,7 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Medkit Merit Badge</t>
+          <t>Tara</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -1743,17 +1811,17 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>Walk It Off, Scout</t>
+          <t>Walk It Off</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>While you have 20+ Injury, climbing and sprinting tire you 25% less.</t>
+          <t>While you have 20+ Injury, climbing and sprinting use 25% less stamina .</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Every injury hurts 20% more.</t>
+          <t>Every injury hurts 10% more.</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr"/>
@@ -1791,13 +1859,17 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Once per biome, when Poison, Spores or Drowsy reaches 35, 20 of it clears at once.</t>
+          <t>Once per biome, press K when Poison, Spores or Drowsy reaches 35 to clear 20 of the worst one.</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr"/>
       <c r="I29" s="6" t="inlineStr"/>
       <c r="J29" s="6" t="inlineStr"/>
-      <c r="K29" s="4" t="inlineStr"/>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>Manual K; clear 20 from the worst Poison/Spores/Drowsy status at 35+, once per biome. Key configurable.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="100" customHeight="1">
       <c r="A30" s="4" t="n">
@@ -1825,7 +1897,7 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>BingBong Flight Insurance</t>
+          <t>BingBong Parachute</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -1835,7 +1907,7 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>You come back with 40 Injury and skip your next card pick.</t>
+          <t>If used, prevents the next card pick.</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr"/>
@@ -1912,7 +1984,7 @@
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>Curse builds up 70% slower.</t>
+          <t>Reviving does not add Curse.</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
@@ -1950,7 +2022,7 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>Tenacity Tincture</t>
+          <t>Mini  Tenacity</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -1988,7 +2060,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -1998,19 +2070,19 @@
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>One extra pocket.</t>
+          <t>All carried weight is cut in half, including your backpack and a carried scout.</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>Everything you carry is 35% heavier.</t>
+          <t>Your third pocket is locked for the rest of the run.</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr"/>
       <c r="J34" s="6" t="inlineStr"/>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>DISABLED: extra pocket is not implemented. If enabled, only the 35% weight penalty works.</t>
+          <t>Now halves total weight and blocks new items in the third pocket; existing items remain retrievable. Enabled by default on a fresh config; previous Enabled=false is preserved.</t>
         </is>
       </c>
     </row>
@@ -2045,10 +2117,14 @@
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>Everything you carry is 20% lighter.</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr"/>
+          <t>Items in your hands weigh 25% less.</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>Items inside your backpack weigh 10% more.</t>
+        </is>
+      </c>
       <c r="I35" s="6" t="inlineStr"/>
       <c r="J35" s="6" t="inlineStr"/>
       <c r="K35" s="4" t="inlineStr"/>
@@ -2126,7 +2202,11 @@
           <t>Once per biome, the first cooked food you eat isn't used up.</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr"/>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>Uncooked food cures hunger 50% less.</t>
+        </is>
+      </c>
       <c r="I37" s="6" t="inlineStr"/>
       <c r="J37" s="6" t="inlineStr"/>
       <c r="K37" s="4" t="inlineStr">
@@ -2204,17 +2284,17 @@
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>Lord of the Spools</t>
+          <t>Balright</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>A free rope spool appears for you at each new campfire.</t>
+          <t>A Balloon Bunch appears for you at the next campfire (once per run).</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>Climbing tires you 8% more.</t>
+          <t>Every stamina use costs 10% more.</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr"/>
@@ -2296,14 +2376,14 @@
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>Your third pocket is locked for the rest of the run.</t>
+          <t>Gain one random, permanent drawback: +15% climbing cost, +15% sprint cost, +20% Injury or +20% Hunger.</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr"/>
       <c r="J41" s="6" t="inlineStr"/>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>Pocket lock keeps items already in the pocket; it blocks new use of that pocket.</t>
+          <t>Two bonus cards and one permanent random penalty. The selected penalty is shown in Current Build and retained in state sync.</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2418,7 @@
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>Near a teammate (6 m), climbing tires you both 15% less.</t>
+          <t>Climbing near a teammate uses 15% less stamina for you both.</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
@@ -2376,7 +2456,7 @@
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>Tara's First Aid Badge</t>
+          <t>First Aid Badge</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
@@ -2431,7 +2511,11 @@
           <t>Carrying a scout feels 35% lighter.</t>
         </is>
       </c>
-      <c r="H44" s="6" t="inlineStr"/>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>While you carry a passed-out scout, their paused death timer drains at 15% of normal speed (or 15% faster if already draining).</t>
+        </is>
+      </c>
       <c r="I44" s="6" t="inlineStr"/>
       <c r="J44" s="6" t="inlineStr"/>
       <c r="K44" s="4" t="inlineStr"/>
@@ -2470,7 +2554,11 @@
           <t>Huddling warms you 35% more, from 35% farther away.</t>
         </is>
       </c>
-      <c r="H45" s="6" t="inlineStr"/>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>With no teammate within 6 m, you get cold 20% faster.</t>
+        </is>
+      </c>
       <c r="I45" s="6" t="inlineStr"/>
       <c r="J45" s="6" t="inlineStr"/>
       <c r="K45" s="4" t="inlineStr"/>
@@ -2506,7 +2594,7 @@
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>The first time you revive a teammate in each biome, you both get 20 extra (yellow) stamina.</t>
+          <t>The first time you revive a teammate in each biome, you both get full extra stamina bar.</t>
         </is>
       </c>
       <c r="H46" s="6" t="inlineStr"/>
@@ -2544,7 +2632,7 @@
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>Long-Distance Uppies</t>
+          <t>You're alright, you're alright</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
@@ -2552,7 +2640,11 @@
           <t>Pull teammates up from 30% farther away.</t>
         </is>
       </c>
-      <c r="H47" s="6" t="inlineStr"/>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>Starting a teammate pull costs you 10 stamina (once per reach).</t>
+        </is>
+      </c>
       <c r="I47" s="6" t="inlineStr"/>
       <c r="J47" s="6" t="inlineStr"/>
       <c r="K47" s="4" t="inlineStr"/>
@@ -2634,7 +2726,11 @@
           <t>Teammates near you (6 m) get stamina back 12% faster.</t>
         </is>
       </c>
-      <c r="H49" s="6" t="inlineStr"/>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>With no teammate within 6 m, every stamina use costs you 10% more.</t>
+        </is>
+      </c>
       <c r="I49" s="6" t="inlineStr"/>
       <c r="J49" s="6" t="inlineStr"/>
       <c r="K49" s="4" t="inlineStr"/>
@@ -2675,7 +2771,7 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>Falls hurt 80% more.</t>
+          <t>Falls hurt 40% more.</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr"/>
@@ -2713,12 +2809,12 @@
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>Get 30 extra (yellow) stamina now, and 20 more at every campfire after.</t>
+          <t>Get 30 extra stamina now, and 20 more at every campfire after.</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>Get 10 Curse now, and 5 more at every campfire after.</t>
+          <t>Get 10 Curse now, and 2 more at every campfire after.</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr"/>
@@ -2756,7 +2852,7 @@
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>Everything you carry is 10% lighter. In each biome, a 65% chance of 25 extra (yellow) stamina.</t>
+          <t>Everything you carry is 10% lighter. In each biome, a 65% chance of 25 extra stamina.</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr">
@@ -2799,17 +2895,21 @@
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>Once per biome, press B for 60 extra (yellow) stamina.</t>
+          <t>Once per biome, press B for 60 extra stamina.</t>
         </is>
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>Using it costs you 25 Injury.</t>
+          <t>Using it costs you 15 Injury.</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr"/>
       <c r="J53" s="6" t="inlineStr"/>
-      <c r="K53" s="4" t="inlineStr"/>
+      <c r="K53" s="4" t="inlineStr">
+        <is>
+          <t>Manual B; spend 15 Injury for 60 bonus stamina, once per biome. Key configurable.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="100" customHeight="1">
       <c r="A54" s="4" t="n">
@@ -2929,7 +3029,7 @@
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>Every injury hurts 75% more.</t>
+          <t>Every injury hurts 50% more.</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr"/>
@@ -3181,7 +3281,11 @@
           <t>You turn to stone 35% slower.</t>
         </is>
       </c>
-      <c r="H62" s="6" t="inlineStr"/>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>Fall damage hurts 15% more</t>
+        </is>
+      </c>
       <c r="I62" s="6" t="inlineStr"/>
       <c r="J62" s="6" t="inlineStr"/>
       <c r="K62" s="4" t="inlineStr"/>
@@ -3212,7 +3316,7 @@
       </c>
       <c r="F63" s="6" t="inlineStr">
         <is>
-          <t>Myres' Fine Print</t>
+          <t>Fine Print</t>
         </is>
       </c>
       <c r="G63" s="6" t="inlineStr">
@@ -3255,7 +3359,7 @@
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>Myres' Favorite Scout</t>
+          <t>Scoutmaster</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr">
@@ -3379,7 +3483,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>[["climbStamina", "mul", 0.88, "always", "self"]]</t>
+          <t>[["climbStamina", "mul", 0.88, "always", "self"], ["sprintStamina", "mul", 1.12, "always", "self"]]</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr"/>
@@ -3421,7 +3525,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>[["slipForce", "mul", 0.65, "always", "self"]]</t>
+          <t>[["coldRate", "mul", 0.65, "climbingColdSurface", "self"], ["coldDecay", "mul", 0.9090909090909091, "always", "self"]]</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr"/>
@@ -3442,7 +3546,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[["climbSpeed", "mul", 0.7, "always", "self"]]</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -3513,7 +3617,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>[["fallInjury", "mul", 0.75, "always", "self"]]</t>
+          <t>[["fallInjury", "mul", 0.75, "always", "self"], ["dynamiteInjury", "mul", 3, "always", "self"]]</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr"/>
@@ -3534,7 +3638,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>[["grabReach", "mul", 1.2, "always", "self"]]</t>
+          <t>[["grabReach", "mul", 1.2, "always", "self"], ["staminaUsage", "mul", 1.1, "always", "self"]]</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr"/>
@@ -3586,7 +3690,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>{"threshold": 0.2, "restore": 0.25}</t>
+          <t>{"threshold": 0.2, "restore": 0.25, "cooldown": 300}</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3705,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>[["sprintStamina", "mul", 0.85, "always", "self"]]</t>
+          <t>[["sprintStamina", "mul", 0.85, "always", "self"], ["climbStamina", "mul", 1.15, "always", "self"]]</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr"/>
@@ -3622,7 +3726,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>[["regenDelay", "add", -0.3, "always", "self"]]</t>
+          <t>[["regenDelay", "add", -0.3, "always", "self"], ["maxStamina", "add", -0.15, "always", "self"]]</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr"/>
@@ -3715,12 +3819,12 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>CampfireBonus</t>
+          <t>CampfireMeal</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>{"bonus": 0.15}</t>
+          <t>{}</t>
         </is>
       </c>
     </row>
@@ -3777,7 +3881,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>[["poisonRate", "mul", 0.65, "always", "self"]]</t>
+          <t>[["poisonRate", "mul", 0.65, "always", "self"], ["heatRate", "mul", 1.25, "always", "self"], ["coldRate", "mul", 1.25, "always", "self"]]</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr"/>
@@ -3819,7 +3923,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>[["thornsRate", "mul", 0.6, "always", "self"]]</t>
+          <t>[["thornsRate", "mul", 0.6, "always", "self"], ["thornRemovalTime", "mul", 2, "always", "self"]]</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
@@ -3840,7 +3944,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>[["heatDecay", "mul", 1.6, "always", "self"]]</t>
+          <t>[["heatDecay", "mul", 1.6, "always", "self"], ["heatRate", "mul", 1.15, "always", "self"]]</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr"/>
@@ -3861,7 +3965,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>[["coldDecay", "mul", 1.6, "always", "self"]]</t>
+          <t>[["coldDecay", "mul", 1.6, "always", "self"], ["coldRate", "mul", 1.15, "always", "self"]]</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
@@ -3882,7 +3986,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>[["climbStamina", "mul", 0.7, "poisonOrSpores20", "self"], ["poisonDecay", "mul", 0.7, "always", "self"], ["sporesDecay", "mul", 0.7, "always", "self"]]</t>
+          <t>[["climbStamina", "mul", 0.6, "poisonAbove20", "self"], ["poisonDecay", "mul", 0.7, "always", "self"]]</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr"/>
@@ -3903,13 +4007,17 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>[["nonFallInjury", "mul", 0.8, "always", "self"]]</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr"/>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>MushroomCycle</t>
+        </is>
+      </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{"interval": 600, "duration": 20, "lowGravity": 1}</t>
         </is>
       </c>
     </row>
@@ -3945,7 +4053,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>[["climbStamina", "mul", 0.75, "injury20", "self"], ["sprintStamina", "mul", 0.75, "injury20", "self"], ["allInjury", "mul", 1.2, "always", "self"]]</t>
+          <t>[["climbStamina", "mul", 0.75, "injury20", "self"], ["sprintStamina", "mul", 0.75, "injury20", "self"], ["allInjury", "mul", 1.1, "always", "self"]]</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr"/>
@@ -4001,7 +4109,7 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>{"injury": 0.4}</t>
+          <t>{}</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4145,7 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>[["curseRate", "mul", 0.3, "always", "self"], ["allInjury", "mul", 1.25, "always", "self"]]</t>
+          <t>[["reviveCurse", "mul", 0, "always", "self"], ["allInjury", "mul", 1.25, "always", "self"]]</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr"/>
@@ -4083,12 +4191,12 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>[["invSlots", "add", 1, "always", "self"], ["itemWeight", "mul", 1.35, "always", "self"]]</t>
+          <t>[["totalWeight", "mul", 0.5, "always", "self"]]</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>PackRat</t>
+          <t>PocketTradeoff</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -4108,7 +4216,7 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>[["itemWeight", "mul", 0.8, "always", "self"]]</t>
+          <t>[["heldItemWeight", "mul", 0.75, "always", "self"], ["backpackItemWeight", "mul", 1.1, "always", "self"]]</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr"/>
@@ -4150,7 +4258,7 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[["uncookedFoodHunger", "mul", 0.5, "always", "self"]]</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -4200,17 +4308,17 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>[["climbStamina", "mul", 1.08, "always", "self"]]</t>
+          <t>[["staminaUsage", "mul", 1.1, "always", "self"]]</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>CampfireSpawn</t>
+          <t>NextCampfireSpawn</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>{"item": 0}</t>
+          <t>{"item": 2}</t>
         </is>
       </c>
     </row>
@@ -4260,7 +4368,7 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>{"bonusCards": 2}</t>
+          <t>{"bonusCards": 2, "climbPenalty": 1.15, "sprintPenalty": 1.15, "injuryPenalty": 1.2, "hungerPenalty": 1.2}</t>
         </is>
       </c>
     </row>
@@ -4317,7 +4425,7 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>[["carryScoutWeight", "mul", 0.65, "always", "self"]]</t>
+          <t>[["carryScoutWeight", "mul", 0.65, "always", "self"], ["carriedDeathRate", "mul", 1.15, "always", "self"]]</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr"/>
@@ -4338,13 +4446,13 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>[["huddleStrength", "mul", 1.35, "always", "self"]]</t>
+          <t>[["huddleStrength", "mul", 1.35, "always", "self"], ["coldRate", "mul", 1.2, "noTeammateNear", "self"]]</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr"/>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{"radius": 6}</t>
         </is>
       </c>
     </row>
@@ -4369,7 +4477,7 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>{"bonus": 0.2}</t>
+          <t>{"bonus": 1}</t>
         </is>
       </c>
     </row>
@@ -4387,10 +4495,14 @@
           <t>[["helpReach", "mul", 1.3, "always", "self"]]</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr"/>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>HelpCost</t>
+        </is>
+      </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{"stamina": 0.1}</t>
         </is>
       </c>
     </row>
@@ -4430,7 +4542,7 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>[["regenRate", "mul", 1.12, "always", "team"]]</t>
+          <t>[["regenRate", "mul", 1.12, "always", "team"], ["staminaUsage", "mul", 1.1, "noTeammateNear", "self"]]</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr"/>
@@ -4451,7 +4563,7 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>[["sprintSpeed", "mul", 1.35, "always", "self"], ["jumpHeight", "mul", 1.25, "always", "self"], ["fallInjury", "mul", 1.8, "always", "self"]]</t>
+          <t>[["sprintSpeed", "mul", 1.35, "always", "self"], ["jumpHeight", "mul", 1.25, "always", "self"], ["fallInjury", "mul", 1.4, "always", "self"]]</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr"/>
@@ -4482,7 +4594,7 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>{"bonusNow": 0.3, "bonusFire": 0.2, "curseNow": 0.1, "curseFire": 0.05}</t>
+          <t>{"bonusNow": 0.3, "bonusFire": 0.2, "curseNow": 0.1, "curseFire": 0.02}</t>
         </is>
       </c>
     </row>
@@ -4532,7 +4644,7 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>{"bonus": 0.6, "injury": 0.25}</t>
+          <t>{"bonus": 0.6, "injury": 0.15}</t>
         </is>
       </c>
     </row>
@@ -4597,7 +4709,7 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>[["maxStamina", "add", 0.4, "always", "self"], ["allInjury", "mul", 1.75, "always", "self"]]</t>
+          <t>[["maxStamina", "add", 0.4, "always", "self"], ["allInjury", "mul", 1.5, "always", "self"]]</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr"/>
@@ -4739,7 +4851,7 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>[["petrifyRate", "mul", 0.65, "always", "self"]]</t>
+          <t>[["petrifyRate", "mul", 0.65, "always", "self"], ["fallInjury", "mul", 1.15, "always", "self"]]</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Campfire Cards 0.6.6: Daddy grabs walls from 40% farther away
- Daddy (LedgeDancer): grabReach x1.4 (was x1.2); card text, README and the
  editable workbook updated. The drawback (all stamina costs +10%) is unchanged.
- Balance version 6 refreshes saved card values once (Enabled kept).

220 unit tests and 5 catalog tests pass, preflight clean, Release build with no
warnings.
</commit_message>
<xml_diff>
--- a/design/editable/card-editing.xlsx
+++ b/design/editable/card-editing.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>PEAK target: 2.6.b. Source: design/cards.json, mod 0.6.5. All 64 cards are included. See card-edit-review.xlsx for your submitted requests and their implementation status.</t>
+          <t>PEAK target: 2.6.b. Source: design/cards.json, mod 0.6.6. All 64 cards are included. See card-edit-review.xlsx for your submitted requests and their implementation status.</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Grab walls from 20% farther away.</t>
+          <t>Grab walls from 40% farther away.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>[["grabReach", "mul", 1.2, "always", "self"], ["staminaUsage", "mul", 1.1, "always", "self"]]</t>
+          <t>[["grabReach", "mul", 1.4, "always", "self"], ["staminaUsage", "mul", 1.1, "always", "self"]]</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Campfire Cards 0.7.1: carry fixes, offer options, full card rebalance
0.6.9: card removals no longer lose the fraction the game's float floor
discards (banked and delivered with the next change; Poison/Spores only on
natural decay), difficulty settings above 100% now apply, and F8 Grant Card
fully restores a card after a rejoin.

0.7.0: Offer Count option (1-10 cards per campfire draw) and a Drawbacks
on/off option, both lobby-synced.

0.7.1: full 64-card rebalance - 42 cards tuned, 3 reworked (Double Down
deals 2 bonus cards and halves the next offer, Cursed Crown charges at most
10 Curse per run, Mountain's Bargain charges 5 Curse once at the sacrifice),
every difficulty tier now defaults to 100%, plus HUD and card-text clarity
fixes (pending Delayed Consequences payments, Double Down toast, Clown
Luggage persistence note, Long Arm base fee wording).
</commit_message>
<xml_diff>
--- a/design/editable/card-editing.xlsx
+++ b/design/editable/card-editing.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>PEAK target: 2.6.b. Source: design/cards.json, mod 0.6.6. All 64 cards are included. See card-edit-review.xlsx for your submitted requests and their implementation status.</t>
+          <t>PEAK target: 2.6.b. Source: design/cards.json, mod 0.7.1. All 64 cards are included. See card-edit-review.xlsx for your submitted requests and their implementation status.</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>Sprinting uses 12% more stamina.</t>
+          <t>Sprinting uses 5% more stamina.</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr"/>
@@ -766,7 +766,7 @@
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>Take 30% more fall Injury.</t>
+          <t>Take 15% more fall Injury.</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr"/>
@@ -807,11 +807,7 @@
           <t>Cold builds 35% slower while climbing blue ice.</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>Warming up takes 10% longer.</t>
-        </is>
-      </c>
+      <c r="H4" s="6" t="inlineStr"/>
       <c r="I4" s="6" t="inlineStr"/>
       <c r="J4" s="6" t="inlineStr"/>
       <c r="K4" s="4" t="inlineStr"/>
@@ -895,7 +891,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Each double jump adds 7.5 Drowsy.</t>
+          <t>Each double jump adds 5 Drowsy.</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr"/>
@@ -981,7 +977,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Dynamite deals 3 times as much Injury.</t>
+          <t>Dynamite deals 50% more Injury.</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr"/>
@@ -1024,7 +1020,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>All stamina costs are 10% higher.</t>
+          <t>All stamina costs are 5% higher.</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr"/>
@@ -1067,7 +1063,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>Hunger builds 35% faster.</t>
+          <t>Hunger builds 15% faster.</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr"/>
@@ -1105,7 +1101,7 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Press {key} below 20 stamina to recover 25. Cooldown: 5 min.</t>
+          <t>Press {key} below 20 stamina to recover 30. Cooldown: 3 min.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr"/>
@@ -1153,7 +1149,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>Climbing uses 15% more stamina.</t>
+          <t>Climbing uses 5% more stamina.</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr"/>
@@ -1191,12 +1187,12 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Stamina regeneration starts 0.3s sooner.</t>
+          <t>Stamina regeneration starts 0.5s sooner.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Lose 15 maximum stamina.</t>
+          <t>Lose 5 maximum stamina.</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr"/>
@@ -1282,7 +1278,7 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>Lose 12.5 maximum stamina.</t>
+          <t>Lose 7.5 maximum stamina.</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr"/>
@@ -1320,7 +1316,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Climb for 3s straight: climbing uses 35% less stamina for the next 1s.</t>
+          <t>Climb for 2s straight: climbing uses 40% less stamina for the next 2s.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr"/>
@@ -1364,7 +1360,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Cooked food removes 25% less Hunger.</t>
+          <t>Cooked food removes 10% less Hunger.</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
@@ -1411,7 +1407,7 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>Cold builds 30% faster.</t>
+          <t>Cold builds 10% faster.</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr"/>
@@ -1454,7 +1450,7 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>Heat builds 30% faster.</t>
+          <t>Heat builds 10% faster.</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr"/>
@@ -1497,7 +1493,7 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>Heat and Cold build 25% faster.</t>
+          <t>Heat and Cold build 10% faster.</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr"/>
@@ -1585,11 +1581,7 @@
           <t>New Thorns add 40% less status, rounded to the nearest whole thorn.</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>Removing Thorns takes twice as long.</t>
-        </is>
-      </c>
+      <c r="H22" s="6" t="inlineStr"/>
       <c r="I22" s="6" t="inlineStr"/>
       <c r="J22" s="6" t="inlineStr"/>
       <c r="K22" s="4" t="inlineStr">
@@ -1634,7 +1626,7 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>Heat builds 15% faster.</t>
+          <t>Heat builds 5% faster.</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr"/>
@@ -1677,7 +1669,7 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>Cold builds 15% faster.</t>
+          <t>Cold builds 5% faster.</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr"/>
@@ -1720,7 +1712,7 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Poison wears off 30% slower.</t>
+          <t>Poison wears off 10% slower.</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
@@ -1801,7 +1793,7 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Healing items remove 25% more Injury from you.</t>
+          <t>Healing removes 25% more Injury from you.</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr"/>
@@ -1849,7 +1841,7 @@
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>Take 10% more Injury.</t>
+          <t>Take 5% more Injury.</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr"/>
@@ -1887,7 +1879,7 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Press {key} at 35+ Poison, Spores or Drowsy to remove 20 from the highest. Once per biome.</t>
+          <t>Press {key} at 25+ Poison, Spores or Drowsy to remove 25 from the highest. Once per biome.</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr"/>
@@ -2019,11 +2011,7 @@
           <t>Reviving does not add Curse.</t>
         </is>
       </c>
-      <c r="H32" s="6" t="inlineStr">
-        <is>
-          <t>Take 25% more Injury.</t>
-        </is>
-      </c>
+      <c r="H32" s="6" t="inlineStr"/>
       <c r="I32" s="6" t="inlineStr"/>
       <c r="J32" s="6" t="inlineStr"/>
       <c r="K32" s="4" t="inlineStr"/>
@@ -2149,12 +2137,12 @@
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>Held items weigh 25% less.</t>
+          <t>Held items weigh 45% less.</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>Backpack contents weigh 10% more.</t>
+          <t>Backpack contents weigh 5% more.</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr"/>
@@ -2236,7 +2224,7 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>Uncooked food removes 50% less Hunger.</t>
+          <t>Uncooked food removes 15% less Hunger.</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr"/>
@@ -2283,7 +2271,7 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>Eating cookable food raw adds 7.5 Poison.</t>
+          <t>Eating cookable food raw adds 5 Poison.</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr"/>
@@ -2324,11 +2312,7 @@
           <t>Get one Balloon Bunch at the next campfire. Once per run.</t>
         </is>
       </c>
-      <c r="H39" s="6" t="inlineStr">
-        <is>
-          <t>All stamina costs are 10% higher.</t>
-        </is>
-      </c>
+      <c r="H39" s="6" t="inlineStr"/>
       <c r="I39" s="6" t="inlineStr"/>
       <c r="J39" s="6" t="inlineStr"/>
       <c r="K39" s="4" t="inlineStr"/>
@@ -2408,7 +2392,7 @@
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>One permanent random penalty: climbing or sprinting cost +15%, Injury +20%, or Hunger buildup +20%.</t>
+          <t>One permanent random penalty: climbing or sprinting cost +10%, Injury +10%, or Hunger buildup +10%. It stays even if you give this card up.</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr"/>
@@ -2450,12 +2434,12 @@
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>You and teammates within 6 m use 15% less climbing stamina.</t>
+          <t>You and teammates within 8 m use 20% less climbing stamina.</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>With no teammate within 6 m, climbing uses 15% more stamina.</t>
+          <t>With no teammate within 8 m, climbing uses 5% more stamina.</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr"/>
@@ -2498,7 +2482,7 @@
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>Healing items used on yourself remove 35% less Injury.</t>
+          <t>Healing items used on yourself remove 15% less Injury.</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr"/>
@@ -2543,11 +2527,7 @@
           <t>Carried scouts weigh 35% less.</t>
         </is>
       </c>
-      <c r="H44" s="6" t="inlineStr">
-        <is>
-          <t>Their paused death timer drains at 15% of normal speed. Already-active timers drain 15% faster.</t>
-        </is>
-      </c>
+      <c r="H44" s="6" t="inlineStr"/>
       <c r="I44" s="6" t="inlineStr"/>
       <c r="J44" s="6" t="inlineStr"/>
       <c r="K44" s="4" t="inlineStr">
@@ -2590,11 +2570,7 @@
           <t>Huddling warms you 35% more, from 35% farther away.</t>
         </is>
       </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>With no teammate within 6 m, Cold builds 20% faster.</t>
-        </is>
-      </c>
+      <c r="H45" s="6" t="inlineStr"/>
       <c r="I45" s="6" t="inlineStr"/>
       <c r="J45" s="6" t="inlineStr"/>
       <c r="K45" s="4" t="inlineStr"/>
@@ -2678,7 +2654,7 @@
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>Starting a pull costs 10 stamina, once per continuous reach.</t>
+          <t>Starting a pull costs a base 5 stamina, once per continuous reach.</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr"/>
@@ -2721,7 +2697,7 @@
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>You take half the prevented Injury, up to 10 per hit.</t>
+          <t>You take a quarter of the prevented Injury, up to 5 per hit.</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr"/>
@@ -2759,14 +2735,10 @@
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>Teammates within 6 m recover stamina 12% faster.</t>
-        </is>
-      </c>
-      <c r="H49" s="6" t="inlineStr">
-        <is>
-          <t>With no teammate within 6 m, all stamina costs are 10% higher.</t>
-        </is>
-      </c>
+          <t>You and teammates within 8 m recover stamina 15% faster.</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr"/>
       <c r="I49" s="6" t="inlineStr"/>
       <c r="J49" s="6" t="inlineStr"/>
       <c r="K49" s="4" t="inlineStr"/>
@@ -2807,7 +2779,7 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>Take 40% more fall Injury.</t>
+          <t>Take 25% more fall Injury.</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr"/>
@@ -2850,7 +2822,7 @@
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>Gain 10 Curse now, then 2 at each later campfire.</t>
+          <t>Gain 5 Curse now, then 1 at each later campfire, up to 10 Curse in total.</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr"/>
@@ -2893,7 +2865,7 @@
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>A failed roll adds 20 Injury instead.</t>
+          <t>A failed roll adds 7.5 Injury instead.</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr"/>
@@ -2983,7 +2955,7 @@
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>Stopping after a boost adds 7.5 Drowsy, at most once every 30s.</t>
+          <t>Stopping after a boost adds 2.5 Drowsy, at most once every 60s.</t>
         </is>
       </c>
       <c r="I54" s="6" t="inlineStr"/>
@@ -3065,7 +3037,7 @@
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>Take 50% more Injury.</t>
+          <t>Take 25% more Injury.</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr"/>
@@ -3108,7 +3080,7 @@
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
-          <t>With a backpack: sprint 15% slower.</t>
+          <t>With a backpack: sprint 5% slower.</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr"/>
@@ -3146,12 +3118,12 @@
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>Immediately gain 1 random bonus card, Common to Rare.</t>
+          <t>Immediately gain 2 random bonus cards, Common to Rare.</t>
         </is>
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>Gain 10 Curse. Your next campfire offers only 1 card.</t>
+          <t>Gain 5 Curse. Your next campfire offers only 2 cards.</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr"/>
@@ -3276,7 +3248,7 @@
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>Lose 15 maximum stamina. The revival leaves 40 Injury.</t>
+          <t>The revival leaves 40 Injury.</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr"/>
@@ -3314,14 +3286,10 @@
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>Petrification builds 35% slower.</t>
-        </is>
-      </c>
-      <c r="H62" s="6" t="inlineStr">
-        <is>
-          <t>Take 15% more fall Injury.</t>
-        </is>
-      </c>
+          <t>Petrification builds 50% slower.</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr"/>
       <c r="I62" s="6" t="inlineStr"/>
       <c r="J62" s="6" t="inlineStr"/>
       <c r="K62" s="4" t="inlineStr"/>
@@ -3362,7 +3330,7 @@
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>Gain 5 Curse at each later campfire.</t>
+          <t>Gain 5 Curse when the sacrifice is made.</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr"/>
@@ -3519,7 +3487,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>[["climbStamina", "mul", 0.88, "always", "self"], ["sprintStamina", "mul", 1.12, "always", "self"]]</t>
+          <t>[["climbStamina", "mul", 0.88, "always", "self"], ["sprintStamina", "mul", 1.05, "always", "self"]]</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr"/>
@@ -3540,7 +3508,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>[["jumpHeight", "mul", 1.3, "always", "self"], ["fallInjury", "mul", 1.3, "always", "self"]]</t>
+          <t>[["jumpHeight", "mul", 1.3, "always", "self"], ["fallInjury", "mul", 1.15, "always", "self"]]</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr"/>
@@ -3561,7 +3529,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>[["coldRate", "mul", 0.65, "climbingColdSurface", "self"], ["coldDecay", "mul", 0.9090909090909091, "always", "self"]]</t>
+          <t>[["coldRate", "mul", 0.65, "climbingColdSurface", "self"]]</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr"/>
@@ -3617,7 +3585,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>{"cooldown": 15, "drowsy": 0.075}</t>
+          <t>{"cooldown": 15, "drowsy": 0.05}</t>
         </is>
       </c>
     </row>
@@ -3653,7 +3621,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>[["fallInjury", "mul", 0.75, "always", "self"], ["dynamiteInjury", "mul", 3, "always", "self"]]</t>
+          <t>[["fallInjury", "mul", 0.75, "always", "self"], ["dynamiteInjury", "mul", 1.5, "always", "self"]]</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr"/>
@@ -3674,7 +3642,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>[["grabReach", "mul", 1.4, "always", "self"], ["staminaUsage", "mul", 1.1, "always", "self"]]</t>
+          <t>[["grabReach", "mul", 1.4, "always", "self"], ["staminaUsage", "mul", 1.05, "always", "self"]]</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr"/>
@@ -3695,7 +3663,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>[["maxStamina", "add", 0.25, "always", "self"], ["hungerRate", "mul", 1.35, "always", "self"]]</t>
+          <t>[["maxStamina", "add", 0.25, "always", "self"], ["hungerRate", "mul", 1.15, "always", "self"]]</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr"/>
@@ -3726,7 +3694,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>{"threshold": 0.2, "restore": 0.25, "cooldown": 300}</t>
+          <t>{"threshold": 0.2, "restore": 0.3, "cooldown": 180}</t>
         </is>
       </c>
     </row>
@@ -3741,7 +3709,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>[["sprintStamina", "mul", 0.85, "always", "self"], ["climbStamina", "mul", 1.15, "always", "self"]]</t>
+          <t>[["sprintStamina", "mul", 0.85, "always", "self"], ["climbStamina", "mul", 1.05, "always", "self"]]</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr"/>
@@ -3762,7 +3730,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>[["regenDelay", "add", -0.3, "always", "self"], ["maxStamina", "add", -0.15, "always", "self"]]</t>
+          <t>[["regenDelay", "add", -0.5, "always", "self"], ["maxStamina", "add", -0.05, "always", "self"]]</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr"/>
@@ -3804,7 +3772,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>[["sprintSpeed", "mul", 1.25, "always", "self"], ["maxStamina", "add", -0.125, "always", "self"]]</t>
+          <t>[["sprintSpeed", "mul", 1.25, "always", "self"], ["maxStamina", "add", -0.075, "always", "self"]]</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr"/>
@@ -3825,7 +3793,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>[["climbStamina", "mul", 0.65, "pulseActive", "self"]]</t>
+          <t>[["climbStamina", "mul", 0.6, "pulseActive", "self"]]</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -3835,7 +3803,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>{"buildup": 3, "boost": 1}</t>
+          <t>{"buildup": 2, "boost": 2}</t>
         </is>
       </c>
     </row>
@@ -3850,7 +3818,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>[["cookedFoodHunger", "mul", 0.75, "always", "self"]]</t>
+          <t>[["cookedFoodHunger", "mul", 0.9, "always", "self"]]</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -3875,7 +3843,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>[["heatRate", "mul", 0.5, "always", "self"], ["coldRate", "mul", 1.3, "always", "self"]]</t>
+          <t>[["heatRate", "mul", 0.5, "always", "self"], ["coldRate", "mul", 1.1, "always", "self"]]</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr"/>
@@ -3896,7 +3864,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>[["coldRate", "mul", 0.5, "always", "self"], ["heatRate", "mul", 1.3, "always", "self"]]</t>
+          <t>[["coldRate", "mul", 0.5, "always", "self"], ["heatRate", "mul", 1.1, "always", "self"]]</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr"/>
@@ -3917,7 +3885,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>[["poisonRate", "mul", 0.65, "always", "self"], ["heatRate", "mul", 1.25, "always", "self"], ["coldRate", "mul", 1.25, "always", "self"]]</t>
+          <t>[["poisonRate", "mul", 0.65, "always", "self"], ["heatRate", "mul", 1.1, "always", "self"], ["coldRate", "mul", 1.1, "always", "self"]]</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr"/>
@@ -3959,7 +3927,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>[["thornsRate", "mul", 0.6, "always", "self"], ["thornRemovalTime", "mul", 2, "always", "self"]]</t>
+          <t>[["thornsRate", "mul", 0.6, "always", "self"]]</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr"/>
@@ -3980,7 +3948,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>[["heatDecay", "mul", 1.6, "always", "self"], ["heatRate", "mul", 1.15, "always", "self"]]</t>
+          <t>[["heatDecay", "mul", 1.6, "always", "self"], ["heatRate", "mul", 1.05, "always", "self"]]</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr"/>
@@ -4001,7 +3969,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>[["coldDecay", "mul", 1.6, "always", "self"], ["coldRate", "mul", 1.15, "always", "self"]]</t>
+          <t>[["coldDecay", "mul", 1.6, "always", "self"], ["coldRate", "mul", 1.05, "always", "self"]]</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
@@ -4022,7 +3990,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>[["climbStamina", "mul", 0.6, "poisonAbove20", "self"], ["poisonDecay", "mul", 0.7, "always", "self"]]</t>
+          <t>[["climbStamina", "mul", 0.6, "poisonAbove20", "self"], ["poisonDecay", "mul", 0.9, "always", "self"]]</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr"/>
@@ -4089,7 +4057,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>[["climbStamina", "mul", 0.75, "injury20", "self"], ["sprintStamina", "mul", 0.75, "injury20", "self"], ["allInjury", "mul", 1.1, "always", "self"]]</t>
+          <t>[["climbStamina", "mul", 0.75, "injury20", "self"], ["sprintStamina", "mul", 0.75, "injury20", "self"], ["allInjury", "mul", 1.05, "always", "self"]]</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr"/>
@@ -4120,7 +4088,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>{"threshold": 0.35, "remove": 0.2}</t>
+          <t>{"threshold": 0.25, "remove": 0.25}</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4149,7 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>[["reviveCurse", "mul", 0, "always", "self"], ["allInjury", "mul", 1.25, "always", "self"]]</t>
+          <t>[["reviveCurse", "mul", 0, "always", "self"]]</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr"/>
@@ -4252,7 +4220,7 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>[["heldItemWeight", "mul", 0.75, "always", "self"], ["backpackItemWeight", "mul", 1.1, "always", "self"]]</t>
+          <t>[["heldItemWeight", "mul", 0.55, "always", "self"], ["backpackItemWeight", "mul", 1.05, "always", "self"]]</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr"/>
@@ -4294,7 +4262,7 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>[["uncookedFoodHunger", "mul", 0.5, "always", "self"]]</t>
+          <t>[["uncookedFoodHunger", "mul", 0.85, "always", "self"]]</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -4329,7 +4297,7 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>{"poison": 0.075}</t>
+          <t>{"poison": 0.05}</t>
         </is>
       </c>
     </row>
@@ -4344,7 +4312,7 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>[["staminaUsage", "mul", 1.1, "always", "self"]]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -4404,7 +4372,7 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>{"bonusCards": 2, "climbPenalty": 1.15, "sprintPenalty": 1.15, "injuryPenalty": 1.2, "hungerPenalty": 1.2}</t>
+          <t>{"bonusCards": 2, "climbPenalty": 1.1, "sprintPenalty": 1.1, "injuryPenalty": 1.1, "hungerPenalty": 1.1}</t>
         </is>
       </c>
     </row>
@@ -4419,13 +4387,13 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>[["climbStamina", "mul", 0.85, "always", "team"], ["climbStamina", "mul", 0.85, "teammateNear", "self"], ["climbStamina", "mul", 1.15, "noTeammateNear", "self"]]</t>
+          <t>[["climbStamina", "mul", 0.8, "always", "team"], ["climbStamina", "mul", 0.8, "teammateNear", "self"], ["climbStamina", "mul", 1.05, "noTeammateNear", "self"]]</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr"/>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>{"radius": 6}</t>
+          <t>{"radius": 8}</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4408,7 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>[["healGiven", "mul", 1.6, "always", "self"], ["healSelfUse", "mul", 0.65, "always", "self"]]</t>
+          <t>[["healGiven", "mul", 1.6, "always", "self"], ["healSelfUse", "mul", 0.85, "always", "self"]]</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr"/>
@@ -4461,7 +4429,7 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>[["carryScoutWeight", "mul", 0.65, "always", "self"], ["carriedDeathRate", "mul", 1.15, "always", "self"]]</t>
+          <t>[["carryScoutWeight", "mul", 0.65, "always", "self"]]</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr"/>
@@ -4482,13 +4450,13 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>[["huddleStrength", "mul", 1.35, "always", "self"], ["coldRate", "mul", 1.2, "noTeammateNear", "self"]]</t>
+          <t>[["huddleStrength", "mul", 1.35, "always", "self"]]</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr"/>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>{"radius": 6}</t>
+          <t>{}</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4506,7 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>{"stamina": 0.1}</t>
+          <t>{"stamina": 0.05}</t>
         </is>
       </c>
     </row>
@@ -4563,7 +4531,7 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>{"radius": 6, "absorb": 0.5, "cap": 0.1}</t>
+          <t>{"radius": 6, "absorb": 0.25, "cap": 0.05}</t>
         </is>
       </c>
     </row>
@@ -4578,13 +4546,13 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>[["regenRate", "mul", 1.12, "always", "team"], ["staminaUsage", "mul", 1.1, "noTeammateNear", "self"]]</t>
+          <t>[["regenRate", "mul", 1.15, "always", "team"], ["regenRate", "mul", 1.15, "teammateNear", "self"]]</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr"/>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>{"radius": 6}</t>
+          <t>{"radius": 8}</t>
         </is>
       </c>
     </row>
@@ -4599,7 +4567,7 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>[["sprintSpeed", "mul", 1.35, "always", "self"], ["jumpHeight", "mul", 1.25, "always", "self"], ["fallInjury", "mul", 1.4, "always", "self"]]</t>
+          <t>[["sprintSpeed", "mul", 1.35, "always", "self"], ["jumpHeight", "mul", 1.25, "always", "self"], ["fallInjury", "mul", 1.25, "always", "self"]]</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr"/>
@@ -4630,7 +4598,7 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>{"bonusNow": 0.3, "bonusFire": 0.2, "curseNow": 0.1, "curseFire": 0.02}</t>
+          <t>{"bonusNow": 0.3, "bonusFire": 0.2, "curseNow": 0.05, "curseFire": 0.01, "curseBudget": 0.1}</t>
         </is>
       </c>
     </row>
@@ -4655,7 +4623,7 @@
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>{"chance": 0.65, "bonus": 0.25, "injury": 0.2}</t>
+          <t>{"chance": 0.65, "bonus": 0.25, "injury": 0.075}</t>
         </is>
       </c>
     </row>
@@ -4705,7 +4673,7 @@
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>{"buildup": 2, "drowsy": 0.075, "cooldown": 30}</t>
+          <t>{"buildup": 2, "drowsy": 0.025, "cooldown": 60}</t>
         </is>
       </c>
     </row>
@@ -4745,7 +4713,7 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>[["maxStamina", "add", 0.4, "always", "self"], ["allInjury", "mul", 1.5, "always", "self"]]</t>
+          <t>[["maxStamina", "add", 0.4, "always", "self"], ["allInjury", "mul", 1.25, "always", "self"]]</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr"/>
@@ -4766,7 +4734,7 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>[["sprintSpeed", "mul", 1.3, "noBackpack", "self"], ["jumpHeight", "mul", 1.2, "noBackpack", "self"], ["sprintSpeed", "mul", 0.85, "wearingBackpack", "self"]]</t>
+          <t>[["sprintSpeed", "mul", 1.3, "noBackpack", "self"], ["jumpHeight", "mul", 1.2, "noBackpack", "self"], ["sprintSpeed", "mul", 0.95, "wearingBackpack", "self"]]</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr"/>
@@ -4797,7 +4765,7 @@
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>{"bonusCards": 1, "curse": 0.1}</t>
+          <t>{"bonusCards": 2, "curse": 0.05, "nextOffer": 2}</t>
         </is>
       </c>
     </row>
@@ -4862,7 +4830,7 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>[["maxStamina", "add", -0.15, "always", "self"]]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -4887,7 +4855,7 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>[["petrifyRate", "mul", 0.65, "always", "self"], ["fallInjury", "mul", 1.15, "always", "self"]]</t>
+          <t>[["petrifyRate", "mul", 0.5, "always", "self"]]</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr"/>
@@ -4918,7 +4886,7 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>{"curseFire": 0.05}</t>
+          <t>{"curse": 0.05}</t>
         </is>
       </c>
     </row>

</xml_diff>